<commit_message>
Corrected Birth display name
Corrected Display name for Birth Acknowledgement within MessageHeader URI values and updated change log
</commit_message>
<xml_diff>
--- a/docs/v3.0.0-preview1/CodeSystem-VRM-MessageHeaderURI-cs.xlsx
+++ b/docs/v3.0.0-preview1/CodeSystem-VRM-MessageHeaderURI-cs.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="155">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-08-11T15:01:09-04:00</t>
+    <t>2025-11-25T14:04:25-05:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -168,6 +168,9 @@
     <t>http://nchs.cdc.gov/birth_acknowledgement</t>
   </si>
   <si>
+    <t>Birth Acknowledgement</t>
+  </si>
+  <si>
     <t>Indicates this is  an  acknowledgement for a birth report</t>
   </si>
   <si>
@@ -282,7 +285,7 @@
     <t>http://nchs.cdc.gov/birth_demographics_coding_update</t>
   </si>
   <si>
-    <t>Bith Parental Demographics Coding Update</t>
+    <t>Birth Parental Demographics Coding Update</t>
   </si>
   <si>
     <t>Indicates that this is an updated demographics coding of a birth report</t>
@@ -420,7 +423,7 @@
     <t>Birth Extraction Error</t>
   </si>
   <si>
-    <t>Indicates that this is an extraction error for a Birth report</t>
+    <t>Indicates that this is an extraction error for a birth report</t>
   </si>
   <si>
     <t>http://nchs.cdc.gov/vrdr_status</t>
@@ -851,10 +854,10 @@
         <v>50</v>
       </c>
       <c r="C5" t="s" s="2">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6">
@@ -862,13 +865,13 @@
         <v>40</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C6" t="s" s="2">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7">
@@ -876,13 +879,13 @@
         <v>40</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C7" t="s" s="2">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D7" t="s" s="2">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8">
@@ -890,13 +893,13 @@
         <v>40</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C8" t="s" s="2">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D8" t="s" s="2">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9">
@@ -904,13 +907,13 @@
         <v>40</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C9" t="s" s="2">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D9" t="s" s="2">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10">
@@ -918,13 +921,13 @@
         <v>40</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C10" t="s" s="2">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D10" t="s" s="2">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11">
@@ -932,13 +935,13 @@
         <v>40</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C11" t="s" s="2">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D11" t="s" s="2">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12">
@@ -946,13 +949,13 @@
         <v>40</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C12" t="s" s="2">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D12" t="s" s="2">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13">
@@ -960,13 +963,13 @@
         <v>40</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C13" t="s" s="2">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D13" t="s" s="2">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="14">
@@ -974,13 +977,13 @@
         <v>40</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C14" t="s" s="2">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D14" t="s" s="2">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="15">
@@ -988,13 +991,13 @@
         <v>40</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C15" t="s" s="2">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D15" t="s" s="2">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="16">
@@ -1002,13 +1005,13 @@
         <v>40</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C16" t="s" s="2">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D16" t="s" s="2">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="17">
@@ -1016,13 +1019,13 @@
         <v>40</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C17" t="s" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D17" t="s" s="2">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="18">
@@ -1030,13 +1033,13 @@
         <v>40</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C18" t="s" s="2">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D18" t="s" s="2">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19">
@@ -1044,13 +1047,13 @@
         <v>40</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C19" t="s" s="2">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D19" t="s" s="2">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="20">
@@ -1058,13 +1061,13 @@
         <v>40</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C20" t="s" s="2">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D20" t="s" s="2">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="21">
@@ -1072,13 +1075,13 @@
         <v>40</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C21" t="s" s="2">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D21" t="s" s="2">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22">
@@ -1086,13 +1089,13 @@
         <v>40</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C22" t="s" s="2">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D22" t="s" s="2">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="23">
@@ -1100,13 +1103,13 @@
         <v>40</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C23" t="s" s="2">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D23" t="s" s="2">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="24">
@@ -1114,13 +1117,13 @@
         <v>40</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C24" t="s" s="2">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D24" t="s" s="2">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="25">
@@ -1128,13 +1131,13 @@
         <v>40</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C25" t="s" s="2">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D25" t="s" s="2">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="26">
@@ -1142,13 +1145,13 @@
         <v>40</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C26" t="s" s="2">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D26" t="s" s="2">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="27">
@@ -1156,13 +1159,13 @@
         <v>40</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C27" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D27" t="s" s="2">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="28">
@@ -1170,13 +1173,13 @@
         <v>40</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C28" t="s" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D28" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="29">
@@ -1184,13 +1187,13 @@
         <v>40</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C29" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D29" t="s" s="2">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="30">
@@ -1198,13 +1201,13 @@
         <v>40</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C30" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D30" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="31">
@@ -1212,13 +1215,13 @@
         <v>40</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C31" t="s" s="2">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D31" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="32">
@@ -1226,13 +1229,13 @@
         <v>40</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C32" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D32" t="s" s="2">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="33">
@@ -1240,13 +1243,13 @@
         <v>40</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C33" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D33" t="s" s="2">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="34">
@@ -1254,13 +1257,13 @@
         <v>40</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C34" t="s" s="2">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D34" t="s" s="2">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="35">
@@ -1268,13 +1271,13 @@
         <v>40</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C35" t="s" s="2">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D35" t="s" s="2">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="36">
@@ -1282,13 +1285,13 @@
         <v>40</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C36" t="s" s="2">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D36" t="s" s="2">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="37">
@@ -1296,13 +1299,13 @@
         <v>40</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C37" t="s" s="2">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D37" t="s" s="2">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="38">
@@ -1310,13 +1313,13 @@
         <v>40</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C38" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D38" t="s" s="2">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="39">
@@ -1324,13 +1327,13 @@
         <v>40</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C39" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D39" t="s" s="2">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>

</xml_diff>